<commit_message>
Added new RDF data schemes and visual schemes for economy-table106-110, fixed XLSX spreadsheet for economy-table108
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table108.xlsx
+++ b/sources/table_normalization/xlsx/economy-table108.xlsx
@@ -78,7 +78,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -94,6 +94,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -166,37 +172,37 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -613,24 +619,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14"/>
-      <c r="D1" s="13" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="14"/>
-      <c r="F1" s="13" t="s">
+      <c r="E1" s="19"/>
+      <c r="F1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="14"/>
+      <c r="G1" s="19"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1">
-      <c r="A2" s="12"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="15" t="s">
         <v>4</v>
       </c>
@@ -645,23 +651,23 @@
       <c r="G2" s="16"/>
     </row>
     <row r="3" spans="1:7" s="1" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A3" s="17"/>
-      <c r="B3" s="18" t="s">
+      <c r="A3" s="18"/>
+      <c r="B3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="14" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>